<commit_message>
PMO TIGRE - atualização da Escala de Trabalho
</commit_message>
<xml_diff>
--- a/Escala de Trabalho.xlsx
+++ b/Escala de Trabalho.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://spotpromo.sharepoint.com/sites/bko.lbasaia/Documentos Compartilhados/PMO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1097" documentId="8_{C9589A86-DEFA-4536-898C-3C99E4F500E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B16963E-CA4F-44F9-BD87-5400652B9100}"/>
+  <xr:revisionPtr revIDLastSave="1104" documentId="8_{C9589A86-DEFA-4536-898C-3C99E4F500E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF43C6DE-7E1A-4FBB-BE34-F29F959D9FD9}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8597F27F-AEEC-4BA4-9237-ED3EB9E49D86}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="983" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="983" uniqueCount="19">
   <si>
     <t>GUSTAVO</t>
   </si>
@@ -94,6 +94,9 @@
   <si>
     <t>SPOT LESTE</t>
   </si>
+  <si>
+    <t>ATESTADO</t>
+  </si>
 </sst>
 </file>
 
@@ -132,7 +135,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -154,6 +157,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -185,7 +194,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -193,11 +202,12 @@
     <xf numFmtId="16" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="279">
+  <dxfs count="245">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -235,6 +245,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -256,36 +276,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -352,6 +342,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -397,46 +407,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <border>
         <left style="thin">
           <color rgb="FF9C0006"/>
@@ -454,21 +424,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -484,21 +454,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -520,6 +490,46 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -596,31 +606,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -652,46 +642,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -728,6 +678,36 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -804,31 +784,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -850,21 +820,31 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -946,21 +926,31 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -982,6 +972,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -1058,6 +1058,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -1114,6 +1124,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -1236,16 +1256,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -1312,6 +1322,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -1322,11 +1342,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1378,6 +1398,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -1444,16 +1474,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -1509,46 +1529,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <border>
         <left style="thin">
           <color rgb="FF9C0006"/>
@@ -1566,6 +1546,26 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -1622,26 +1622,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -1652,21 +1632,51 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1688,21 +1698,31 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1718,21 +1738,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1754,26 +1764,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -1784,11 +1774,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1820,31 +1810,31 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1870,11 +1860,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1925,26 +1925,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <border>
         <left style="thin">
           <color rgb="FF9C0006"/>
@@ -1962,21 +1942,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1992,21 +1972,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2028,31 +2008,41 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2084,11 +2074,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2104,21 +2094,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2140,11 +2130,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2160,21 +2160,61 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2205,36 +2245,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <border>
         <left style="thin">
           <color rgb="FF9C0006"/>
@@ -2252,31 +2262,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2292,21 +2292,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2328,11 +2328,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2353,26 +2363,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2394,21 +2384,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2419,6 +2409,46 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2470,41 +2500,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2536,6 +2536,56 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -2546,21 +2596,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2602,31 +2642,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2648,21 +2668,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2678,21 +2698,51 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2714,11 +2764,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2734,21 +2794,42 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2770,31 +2851,31 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2805,459 +2886,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF9C0006"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF9C0006"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF9C0006"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF9C0006"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF9C0006"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF9C0006"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF9C0006"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF9C0006"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF9C0006"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF9C0006"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF9C0006"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF9C0006"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF9C0006"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF9C0006"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF9C0006"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF9C0006"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF9C0006"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF9C0006"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF9C0006"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF9C0006"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF9C0006"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF9C0006"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF9C0006"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF9C0006"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF9C0006"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF9C0006"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF9C0006"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF9C0006"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3605,6 +3233,7 @@
     <col min="12" max="12" width="13.88671875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="13.109375" bestFit="1" customWidth="1"/>
     <col min="14" max="15" width="1.77734375" customWidth="1"/>
+    <col min="16" max="17" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="21" max="22" width="1.44140625" customWidth="1"/>
     <col min="26" max="26" width="7.21875" bestFit="1" customWidth="1"/>
@@ -5367,11 +4996,11 @@
       <c r="M50" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="P50" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="Q50" s="3" t="s">
-        <v>9</v>
+      <c r="P50" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q50" s="7" t="s">
+        <v>18</v>
       </c>
       <c r="R50" s="3" t="s">
         <v>16</v>
@@ -5380,7 +5009,7 @@
         <v>9</v>
       </c>
       <c r="T50" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="W50" s="3" t="s">
         <v>10</v>
@@ -7064,972 +6693,858 @@
     </row>
   </sheetData>
   <autoFilter ref="A16:A24" xr:uid="{FA93638E-3964-4B9F-B2A5-0DADAAE5D49F}"/>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="cellIs" dxfId="244" priority="628" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="243" priority="627" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="242" priority="629" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A4:F12">
+    <cfRule type="cellIs" dxfId="241" priority="621" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="240" priority="620" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A1:XFD1048576">
-    <cfRule type="cellIs" dxfId="278" priority="67" operator="equal">
+    <cfRule type="cellIs" dxfId="239" priority="75" operator="equal">
+      <formula>"CAMPO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="238" priority="68" operator="equal">
+      <formula>"PLATINA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="237" priority="67" operator="equal">
       <formula>"SPOT LESTE"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="277" priority="68" operator="equal">
-      <formula>"PLATINA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="276" priority="75" operator="equal">
-      <formula>"CAMPO"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="275" priority="82" operator="equal">
+    <cfRule type="cellIs" dxfId="236" priority="82" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="cellIs" dxfId="274" priority="627" operator="equal">
+  <conditionalFormatting sqref="B50">
+    <cfRule type="cellIs" dxfId="235" priority="74" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="234" priority="73" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="233" priority="72" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="273" priority="628" operator="equal">
+    <cfRule type="cellIs" dxfId="232" priority="71" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="231" priority="70" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="230" priority="69" operator="equal">
+      <formula>"PLATINA 33B"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B47:E47">
+    <cfRule type="cellIs" dxfId="229" priority="422" operator="equal">
+      <formula>"PLATINA 33B"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B4:F12">
+    <cfRule type="cellIs" dxfId="228" priority="623" operator="equal">
       <formula>"HOME"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="272" priority="629" operator="equal">
+    <cfRule type="cellIs" dxfId="227" priority="622" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="226" priority="624" operator="equal">
       <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:A12">
-    <cfRule type="cellIs" dxfId="271" priority="625" operator="equal">
+  <conditionalFormatting sqref="B26:F43">
+    <cfRule type="cellIs" dxfId="225" priority="461" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="224" priority="460" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="223" priority="459" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="222" priority="458" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="270" priority="626" operator="equal">
-      <formula>"FÉRIAS"</formula>
+    <cfRule type="cellIs" dxfId="221" priority="462" operator="equal">
+      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27:F34">
-    <cfRule type="cellIs" dxfId="269" priority="613" operator="equal">
+    <cfRule type="cellIs" dxfId="220" priority="613" operator="equal">
       <formula>"PLATINA 33B"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B4:F12">
-    <cfRule type="cellIs" dxfId="268" priority="620" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="267" priority="621" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="266" priority="622" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="265" priority="623" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="264" priority="624" operator="equal">
-      <formula>"SPOT"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B50">
-    <cfRule type="cellIs" dxfId="263" priority="69" operator="equal">
-      <formula>"PLATINA 33B"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="262" priority="70" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="261" priority="71" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="260" priority="72" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="259" priority="73" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="258" priority="74" operator="equal">
-      <formula>"SPOT"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B47:E47">
-    <cfRule type="cellIs" dxfId="257" priority="422" operator="equal">
-      <formula>"PLATINA 33B"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B26:F34">
-    <cfRule type="cellIs" dxfId="256" priority="615" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="255" priority="616" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="254" priority="617" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="253" priority="618" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="252" priority="619" operator="equal">
-      <formula>"SPOT"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B35:F43">
-    <cfRule type="cellIs" dxfId="251" priority="458" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="250" priority="459" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="249" priority="460" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="248" priority="461" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="247" priority="462" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B36:F43">
-    <cfRule type="cellIs" dxfId="246" priority="457" operator="equal">
+    <cfRule type="cellIs" dxfId="219" priority="457" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B46:F46 B47:E47">
-    <cfRule type="cellIs" dxfId="245" priority="423" operator="equal">
+    <cfRule type="cellIs" dxfId="218" priority="423" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="244" priority="424" operator="equal">
+    <cfRule type="cellIs" dxfId="217" priority="427" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="216" priority="426" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="215" priority="425" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="214" priority="424" operator="equal">
       <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="243" priority="425" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="242" priority="426" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="241" priority="427" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B48:F54">
-    <cfRule type="cellIs" dxfId="240" priority="43" operator="equal">
+    <cfRule type="cellIs" dxfId="213" priority="45" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="212" priority="46" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="211" priority="48" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="210" priority="43" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="239" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="209" priority="44" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="238" priority="45" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="237" priority="46" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="236" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="208" priority="47" operator="equal">
       <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="235" priority="48" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B58:F65">
-    <cfRule type="cellIs" dxfId="234" priority="339" operator="equal">
+    <cfRule type="cellIs" dxfId="207" priority="339" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69:F76">
-    <cfRule type="cellIs" dxfId="233" priority="173" operator="equal">
+    <cfRule type="cellIs" dxfId="206" priority="174" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="205" priority="176" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="204" priority="175" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="203" priority="173" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="232" priority="174" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="231" priority="175" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="230" priority="176" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="229" priority="177" operator="equal">
+    <cfRule type="cellIs" dxfId="202" priority="178" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="201" priority="177" operator="equal">
       <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="228" priority="178" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B68:AH68">
-    <cfRule type="cellIs" dxfId="227" priority="245" operator="equal">
+    <cfRule type="cellIs" dxfId="200" priority="249" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="199" priority="248" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="198" priority="247" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="197" priority="246" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="196" priority="245" operator="equal">
       <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="226" priority="246" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="225" priority="247" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="224" priority="248" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="223" priority="249" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F47:F54">
-    <cfRule type="cellIs" dxfId="222" priority="375" operator="equal">
+    <cfRule type="cellIs" dxfId="195" priority="379" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="194" priority="380" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="193" priority="378" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="192" priority="377" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="191" priority="376" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="190" priority="375" operator="equal">
       <formula>"PLATINA 33B"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="221" priority="376" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="220" priority="377" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="219" priority="378" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="218" priority="379" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="217" priority="380" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F59:F65">
-    <cfRule type="cellIs" dxfId="216" priority="304" operator="equal">
+    <cfRule type="cellIs" dxfId="189" priority="309" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="188" priority="308" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="187" priority="307" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="186" priority="306" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="185" priority="305" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="184" priority="304" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="215" priority="305" operator="equal">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I26:M43">
+    <cfRule type="cellIs" dxfId="183" priority="452" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="214" priority="306" operator="equal">
+    <cfRule type="cellIs" dxfId="182" priority="455" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="181" priority="454" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="180" priority="456" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="179" priority="453" operator="equal">
       <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="213" priority="307" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="212" priority="308" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="211" priority="309" operator="equal">
-      <formula>"SPOT"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I26:M34">
-    <cfRule type="cellIs" dxfId="210" priority="608" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="209" priority="609" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="208" priority="610" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="207" priority="611" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="206" priority="612" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I27:M34">
-    <cfRule type="cellIs" dxfId="205" priority="607" operator="equal">
+    <cfRule type="cellIs" dxfId="178" priority="607" operator="equal">
       <formula>"PLATINA 33B"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I35:M43">
-    <cfRule type="cellIs" dxfId="204" priority="452" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="203" priority="453" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="202" priority="454" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="201" priority="455" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="200" priority="456" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I36:M43">
-    <cfRule type="cellIs" dxfId="199" priority="451" operator="equal">
+    <cfRule type="cellIs" dxfId="177" priority="451" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I46:M54">
-    <cfRule type="cellIs" dxfId="198" priority="417" operator="equal">
+    <cfRule type="cellIs" dxfId="176" priority="420" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="175" priority="419" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="174" priority="418" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="173" priority="417" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="197" priority="418" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="196" priority="419" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="195" priority="420" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="194" priority="421" operator="equal">
+    <cfRule type="cellIs" dxfId="172" priority="421" operator="equal">
       <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I47:M54">
-    <cfRule type="cellIs" dxfId="193" priority="416" operator="equal">
+    <cfRule type="cellIs" dxfId="171" priority="416" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I57:M65">
-    <cfRule type="cellIs" dxfId="192" priority="334" operator="equal">
+    <cfRule type="cellIs" dxfId="170" priority="337" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="169" priority="335" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="168" priority="334" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="191" priority="335" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="190" priority="336" operator="equal">
+    <cfRule type="cellIs" dxfId="167" priority="336" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="189" priority="337" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="188" priority="338" operator="equal">
+    <cfRule type="cellIs" dxfId="166" priority="338" operator="equal">
       <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I58:M65">
-    <cfRule type="cellIs" dxfId="187" priority="333" operator="equal">
+    <cfRule type="cellIs" dxfId="165" priority="333" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I69:M76">
-    <cfRule type="cellIs" dxfId="186" priority="238" operator="equal">
+    <cfRule type="cellIs" dxfId="164" priority="241" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="163" priority="240" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="162" priority="239" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="161" priority="243" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="160" priority="238" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="185" priority="239" operator="equal">
+    <cfRule type="cellIs" dxfId="159" priority="242" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J50">
+    <cfRule type="cellIs" dxfId="158" priority="40" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="157" priority="39" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="156" priority="38" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="184" priority="240" operator="equal">
+    <cfRule type="cellIs" dxfId="155" priority="41" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="154" priority="42" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="153" priority="37" operator="equal">
+      <formula>"PLATINA 33B"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J52">
+    <cfRule type="cellIs" dxfId="152" priority="32" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="151" priority="31" operator="equal">
+      <formula>"PLATINA 33B"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="150" priority="36" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="149" priority="34" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="148" priority="35" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="147" priority="33" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="183" priority="241" operator="equal">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L47:L48">
+    <cfRule type="cellIs" dxfId="146" priority="19" operator="equal">
+      <formula>"PLATINA 33B"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="145" priority="22" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="182" priority="242" operator="equal">
+    <cfRule type="cellIs" dxfId="144" priority="20" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="143" priority="21" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="142" priority="24" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="141" priority="23" operator="equal">
       <formula>"HOME"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="181" priority="243" operator="equal">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M49">
+    <cfRule type="cellIs" dxfId="140" priority="14" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="139" priority="13" operator="equal">
+      <formula>"PLATINA 33B"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="138" priority="17" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="137" priority="16" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="136" priority="18" operator="equal">
       <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="135" priority="15" operator="equal">
+      <formula>"FÉRIAS"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P36:Q43">
-    <cfRule type="cellIs" dxfId="180" priority="440" operator="equal">
+    <cfRule type="cellIs" dxfId="134" priority="440" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="179" priority="441" operator="equal">
+    <cfRule type="cellIs" dxfId="133" priority="444" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="132" priority="441" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="178" priority="442" operator="equal">
+    <cfRule type="cellIs" dxfId="131" priority="443" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="130" priority="442" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="177" priority="443" operator="equal">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P54:Q54 P47:Q52">
+    <cfRule type="cellIs" dxfId="129" priority="409" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="128" priority="408" operator="equal">
       <formula>"HOME"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="176" priority="444" operator="equal">
-      <formula>"SPOT"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P47:Q52 P54:Q54">
-    <cfRule type="cellIs" dxfId="175" priority="405" operator="equal">
+    <cfRule type="cellIs" dxfId="127" priority="405" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="174" priority="406" operator="equal">
+    <cfRule type="cellIs" dxfId="126" priority="406" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="173" priority="407" operator="equal">
+    <cfRule type="cellIs" dxfId="125" priority="407" operator="equal">
       <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="172" priority="408" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="171" priority="409" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P58:Q65">
-    <cfRule type="cellIs" dxfId="170" priority="322" operator="equal">
+    <cfRule type="cellIs" dxfId="124" priority="325" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="123" priority="326" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="122" priority="324" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="121" priority="323" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="120" priority="322" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="169" priority="323" operator="equal">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P26:T43">
+    <cfRule type="cellIs" dxfId="119" priority="468" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="118" priority="464" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="117" priority="465" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="168" priority="324" operator="equal">
+    <cfRule type="cellIs" dxfId="116" priority="466" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="167" priority="325" operator="equal">
+    <cfRule type="cellIs" dxfId="115" priority="467" operator="equal">
       <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="166" priority="326" operator="equal">
-      <formula>"SPOT"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P26:T34">
-    <cfRule type="cellIs" dxfId="165" priority="524" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="164" priority="525" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="163" priority="526" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="162" priority="527" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="161" priority="528" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P27:T34">
-    <cfRule type="cellIs" dxfId="160" priority="523" operator="equal">
+    <cfRule type="cellIs" dxfId="114" priority="523" operator="equal">
       <formula>"PLATINA 33B"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P35:T43">
-    <cfRule type="cellIs" dxfId="159" priority="464" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="158" priority="465" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="157" priority="466" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="156" priority="467" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="155" priority="468" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P36:T43">
-    <cfRule type="cellIs" dxfId="154" priority="463" operator="equal">
+    <cfRule type="cellIs" dxfId="113" priority="463" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P46:T54">
-    <cfRule type="cellIs" dxfId="153" priority="132" operator="equal">
+    <cfRule type="cellIs" dxfId="112" priority="132" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="152" priority="133" operator="equal">
+    <cfRule type="cellIs" dxfId="111" priority="133" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="151" priority="134" operator="equal">
+    <cfRule type="cellIs" dxfId="110" priority="134" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="150" priority="135" operator="equal">
+    <cfRule type="cellIs" dxfId="109" priority="135" operator="equal">
       <formula>"HOME"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="149" priority="136" operator="equal">
+    <cfRule type="cellIs" dxfId="108" priority="136" operator="equal">
       <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P47:T54">
-    <cfRule type="cellIs" dxfId="148" priority="131" operator="equal">
+    <cfRule type="cellIs" dxfId="107" priority="131" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P58:T65">
-    <cfRule type="cellIs" dxfId="147" priority="345" operator="equal">
+    <cfRule type="cellIs" dxfId="106" priority="345" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P69:T76">
-    <cfRule type="cellIs" dxfId="146" priority="227" operator="equal">
+    <cfRule type="cellIs" dxfId="105" priority="227" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="145" priority="228" operator="equal">
+    <cfRule type="cellIs" dxfId="104" priority="228" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="144" priority="229" operator="equal">
+    <cfRule type="cellIs" dxfId="103" priority="231" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="102" priority="230" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="101" priority="229" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="143" priority="230" operator="equal">
+    <cfRule type="cellIs" dxfId="100" priority="250" operator="equal">
+      <formula>"PLATINA 33B"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R48:R49">
+    <cfRule type="cellIs" dxfId="99" priority="1" operator="equal">
+      <formula>"PLATINA 33B"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="98" priority="2" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="97" priority="3" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="96" priority="4" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="95" priority="5" operator="equal">
       <formula>"HOME"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="142" priority="231" operator="equal">
+    <cfRule type="cellIs" dxfId="94" priority="6" operator="equal">
       <formula>"SPOT"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="141" priority="250" operator="equal">
-      <formula>"PLATINA 33B"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W47:W54">
-    <cfRule type="cellIs" dxfId="140" priority="84" operator="equal">
+    <cfRule type="cellIs" dxfId="93" priority="84" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="139" priority="85" operator="equal">
+    <cfRule type="cellIs" dxfId="92" priority="85" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="138" priority="86" operator="equal">
+    <cfRule type="cellIs" dxfId="91" priority="86" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="137" priority="87" operator="equal">
+    <cfRule type="cellIs" dxfId="90" priority="87" operator="equal">
       <formula>"HOME"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="136" priority="88" operator="equal">
+    <cfRule type="cellIs" dxfId="89" priority="88" operator="equal">
       <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W36:X36 W37:Y43">
-    <cfRule type="cellIs" dxfId="135" priority="499" operator="equal">
+    <cfRule type="cellIs" dxfId="88" priority="499" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W26:AA34">
-    <cfRule type="cellIs" dxfId="134" priority="596" operator="equal">
+  <conditionalFormatting sqref="W26:AA35 W36:X36 W37:Y43">
+    <cfRule type="cellIs" dxfId="87" priority="500" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="133" priority="597" operator="equal">
+    <cfRule type="cellIs" dxfId="86" priority="501" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="132" priority="598" operator="equal">
+    <cfRule type="cellIs" dxfId="85" priority="502" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="131" priority="599" operator="equal">
+    <cfRule type="cellIs" dxfId="84" priority="503" operator="equal">
       <formula>"HOME"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="130" priority="600" operator="equal">
+    <cfRule type="cellIs" dxfId="83" priority="504" operator="equal">
       <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W27:AA34">
-    <cfRule type="cellIs" dxfId="129" priority="595" operator="equal">
+    <cfRule type="cellIs" dxfId="82" priority="595" operator="equal">
       <formula>"PLATINA 33B"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W35:AA35 W36:X36 W37:Y43">
-    <cfRule type="cellIs" dxfId="128" priority="500" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="127" priority="501" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="126" priority="502" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="125" priority="503" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="124" priority="504" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W46:AA54">
-    <cfRule type="cellIs" dxfId="123" priority="126" operator="equal">
+    <cfRule type="cellIs" dxfId="81" priority="126" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="122" priority="127" operator="equal">
+    <cfRule type="cellIs" dxfId="80" priority="127" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="121" priority="128" operator="equal">
+    <cfRule type="cellIs" dxfId="79" priority="128" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="120" priority="129" operator="equal">
+    <cfRule type="cellIs" dxfId="78" priority="129" operator="equal">
       <formula>"HOME"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="119" priority="130" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="130" operator="equal">
       <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W47:AA54">
-    <cfRule type="cellIs" dxfId="118" priority="76" operator="equal">
+    <cfRule type="cellIs" dxfId="76" priority="76" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W57:AA65">
-    <cfRule type="cellIs" dxfId="117" priority="263" operator="equal">
+    <cfRule type="cellIs" dxfId="75" priority="267" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="74" priority="263" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="116" priority="264" operator="equal">
+    <cfRule type="cellIs" dxfId="73" priority="264" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="115" priority="265" operator="equal">
+    <cfRule type="cellIs" dxfId="72" priority="265" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="114" priority="266" operator="equal">
+    <cfRule type="cellIs" dxfId="71" priority="266" operator="equal">
       <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="113" priority="267" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W58:AA65">
-    <cfRule type="cellIs" dxfId="112" priority="262" operator="equal">
+    <cfRule type="cellIs" dxfId="70" priority="262" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W69:AA76">
-    <cfRule type="cellIs" dxfId="111" priority="209" operator="equal">
+    <cfRule type="cellIs" dxfId="69" priority="211" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="68" priority="210" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="67" priority="214" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="66" priority="212" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="65" priority="209" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="110" priority="210" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="109" priority="211" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="108" priority="212" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="107" priority="213" operator="equal">
+    <cfRule type="cellIs" dxfId="64" priority="213" operator="equal">
       <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="106" priority="214" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Y48:Y52">
-    <cfRule type="cellIs" dxfId="105" priority="434" operator="equal">
+    <cfRule type="cellIs" dxfId="63" priority="439" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="62" priority="434" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="104" priority="435" operator="equal">
+    <cfRule type="cellIs" dxfId="61" priority="435" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="103" priority="436" operator="equal">
+    <cfRule type="cellIs" dxfId="60" priority="436" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="102" priority="437" operator="equal">
+    <cfRule type="cellIs" dxfId="59" priority="437" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="101" priority="438" operator="equal">
+    <cfRule type="cellIs" dxfId="58" priority="438" operator="equal">
       <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="439" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Y59:Y65">
-    <cfRule type="cellIs" dxfId="99" priority="351" operator="equal">
+    <cfRule type="cellIs" dxfId="57" priority="355" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="56" priority="354" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="55" priority="353" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="54" priority="352" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="53" priority="351" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="98" priority="352" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="97" priority="353" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="96" priority="354" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="95" priority="355" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="94" priority="356" operator="equal">
+    <cfRule type="cellIs" dxfId="52" priority="356" operator="equal">
       <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Y70:Y76">
-    <cfRule type="cellIs" dxfId="93" priority="256" operator="equal">
+    <cfRule type="cellIs" dxfId="51" priority="261" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="50" priority="256" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="92" priority="257" operator="equal">
+    <cfRule type="cellIs" dxfId="49" priority="257" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="91" priority="258" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="258" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="259" operator="equal">
+    <cfRule type="cellIs" dxfId="47" priority="259" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="89" priority="260" operator="equal">
+    <cfRule type="cellIs" dxfId="46" priority="260" operator="equal">
       <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="261" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Y36:AA43">
-    <cfRule type="cellIs" dxfId="87" priority="445" operator="equal">
+    <cfRule type="cellIs" dxfId="45" priority="450" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="44" priority="449" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="43" priority="448" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="42" priority="447" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="41" priority="445" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="86" priority="446" operator="equal">
+    <cfRule type="cellIs" dxfId="40" priority="446" operator="equal">
       <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="85" priority="447" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="448" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="83" priority="449" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="450" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z47:Z54">
-    <cfRule type="cellIs" dxfId="81" priority="77" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="79" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="38" priority="77" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="80" priority="78" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="78" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="79" priority="79" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="80" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="80" operator="equal">
       <formula>"HOME"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="77" priority="81" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="81" operator="equal">
       <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD58:AE58 AD59:AF65">
-    <cfRule type="cellIs" dxfId="76" priority="316" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="317" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="33" priority="318" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="32" priority="319" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="31" priority="320" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="321" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="29" priority="316" operator="equal">
       <formula>"PLATINA 33B"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="75" priority="317" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="74" priority="318" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="73" priority="319" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="320" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="71" priority="321" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD46:AH54">
-    <cfRule type="cellIs" dxfId="70" priority="50" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="54" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="27" priority="53" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="26" priority="52" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="25" priority="51" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="50" operator="equal">
       <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="69" priority="51" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="68" priority="52" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="67" priority="53" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="54" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD47:AH54">
-    <cfRule type="cellIs" dxfId="65" priority="49" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="49" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD57:AH57 B57:F65 P57:T65">
-    <cfRule type="cellIs" dxfId="64" priority="340" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="344" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="343" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="20" priority="342" operator="equal">
+      <formula>"FOLGA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="341" operator="equal">
+      <formula>"FÉRIAS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="18" priority="340" operator="equal">
       <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="63" priority="341" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="62" priority="342" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="343" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="344" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD69:AH76">
-    <cfRule type="cellIs" dxfId="59" priority="185" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="185" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="186" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="186" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="187" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="187" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="188" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="188" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="189" operator="equal">
+    <cfRule type="cellIs" dxfId="13" priority="189" operator="equal">
       <formula>"HOME"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="190" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="190" operator="equal">
       <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF70:AF76">
-    <cfRule type="cellIs" dxfId="53" priority="203" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="207" operator="equal">
+      <formula>"HOME"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="208" operator="equal">
+      <formula>"SPOT"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="203" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="204" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="204" operator="equal">
       <formula>"VIAGEM"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="205" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="205" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="206" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="206" operator="equal">
       <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="49" priority="207" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="208" operator="equal">
-      <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF58:AH65">
-    <cfRule type="cellIs" dxfId="47" priority="310" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="311" operator="equal">
+      <formula>"VIAGEM"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="310" operator="equal">
       <formula>"PLATINA 33B"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="311" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="312" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="312" operator="equal">
       <formula>"FÉRIAS"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="313" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="313" operator="equal">
       <formula>"FOLGA"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="314" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="314" operator="equal">
       <formula>"HOME"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="315" operator="equal">
-      <formula>"SPOT"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J50">
-    <cfRule type="cellIs" dxfId="41" priority="37" operator="equal">
-      <formula>"PLATINA 33B"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="38" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="39" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="40" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="41" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="42" operator="equal">
-      <formula>"SPOT"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J52">
-    <cfRule type="cellIs" dxfId="35" priority="31" operator="equal">
-      <formula>"PLATINA 33B"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="32" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="33" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="34" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="35" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="36" operator="equal">
-      <formula>"SPOT"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L48">
-    <cfRule type="cellIs" dxfId="29" priority="25" operator="equal">
-      <formula>"PLATINA 33B"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="26" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="27" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="28" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="29" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="30" operator="equal">
-      <formula>"SPOT"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L47">
-    <cfRule type="cellIs" dxfId="23" priority="19" operator="equal">
-      <formula>"PLATINA 33B"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="20" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="21" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="22" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="23" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="24" operator="equal">
-      <formula>"SPOT"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M49">
-    <cfRule type="cellIs" dxfId="17" priority="13" operator="equal">
-      <formula>"PLATINA 33B"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="14" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="15" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="16" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="17" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="18" operator="equal">
-      <formula>"SPOT"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R49">
-    <cfRule type="cellIs" dxfId="11" priority="7" operator="equal">
-      <formula>"PLATINA 33B"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="8" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="10" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="11" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="12" operator="equal">
-      <formula>"SPOT"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R48">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
-      <formula>"PLATINA 33B"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
-      <formula>"VIAGEM"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
-      <formula>"FÉRIAS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
-      <formula>"FOLGA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="5" operator="equal">
-      <formula>"HOME"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="315" operator="equal">
       <formula>"SPOT"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8039,26 +7554,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e69c21a7-acf8-4fa1-a5df-4dc7c803cbc8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d337ff45-b2f2-4aee-a0da-7b5a3bfb7c3d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C0248C8800EF904C9DD7E4C547A51745" ma:contentTypeVersion="16" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="99cce447bb6f5efd32e9ce5f489bef41">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e69c21a7-acf8-4fa1-a5df-4dc7c803cbc8" xmlns:ns3="d337ff45-b2f2-4aee-a0da-7b5a3bfb7c3d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4a9ec8dda6a39005fb0ea9e750809ba0" ns2:_="" ns3:_="">
     <xsd:import namespace="e69c21a7-acf8-4fa1-a5df-4dc7c803cbc8"/>
@@ -8299,26 +7794,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{09527016-607A-4F07-A328-80E579B68BCB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="e69c21a7-acf8-4fa1-a5df-4dc7c803cbc8"/>
-    <ds:schemaRef ds:uri="d337ff45-b2f2-4aee-a0da-7b5a3bfb7c3d"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27FD16DC-C657-454C-BC2E-356661B1CA7F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e69c21a7-acf8-4fa1-a5df-4dc7c803cbc8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d337ff45-b2f2-4aee-a0da-7b5a3bfb7c3d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D068290E-986D-4310-B08B-7FF0E4AECC6B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8335,4 +7831,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{27FD16DC-C657-454C-BC2E-356661B1CA7F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{09527016-607A-4F07-A328-80E579B68BCB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e69c21a7-acf8-4fa1-a5df-4dc7c803cbc8"/>
+    <ds:schemaRef ds:uri="d337ff45-b2f2-4aee-a0da-7b5a3bfb7c3d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>